<commit_message>
situation familiale not entring problem fixed 17-02-2025
</commit_message>
<xml_diff>
--- a/sourceEnq/Template-Fr.xlsx
+++ b/sourceEnq/Template-Fr.xlsx
@@ -101,9 +101,6 @@
     <t>Adresse</t>
   </si>
   <si>
-    <t xml:space="preserve">Situation Familiale </t>
-  </si>
-  <si>
     <t>Date de naissance Conjoin</t>
   </si>
   <si>
@@ -126,6 +123,9 @@
   </si>
   <si>
     <t>Catégorie ( Plus/ Moin)</t>
+  </si>
+  <si>
+    <t>Situation Familiale</t>
   </si>
 </sst>
 </file>
@@ -965,7 +965,7 @@
         <v>23</v>
       </c>
       <c r="P1" s="58" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="Q1" s="58" t="s">
         <v>21</v>
@@ -977,28 +977,28 @@
         <v>11</v>
       </c>
       <c r="T1" s="63" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="U1" s="58" t="s">
+      <c r="V1" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="V1" s="58" t="s">
+      <c r="W1" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="W1" s="64" t="s">
+      <c r="X1" s="57" t="s">
         <v>28</v>
       </c>
-      <c r="X1" s="57" t="s">
+      <c r="Y1" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="Y1" s="61" t="s">
+      <c r="Z1" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="Z1" s="57" t="s">
+      <c r="AA1" s="57" t="s">
         <v>31</v>
-      </c>
-      <c r="AA1" s="57" t="s">
-        <v>32</v>
       </c>
       <c r="AB1" s="57" t="s">
         <v>16</v>

</xml_diff>